<commit_message>
Update automático: 2026-05-03 20:13
</commit_message>
<xml_diff>
--- a/HISTORICO.xlsx
+++ b/HISTORICO.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V9"/>
+  <dimension ref="A1:V11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1081,17 +1081,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="P8" t="inlineStr"/>
-      <c r="Q8" t="inlineStr"/>
-      <c r="R8" t="inlineStr"/>
-      <c r="S8" t="inlineStr"/>
-      <c r="T8" t="inlineStr"/>
       <c r="U8" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="V8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1154,9 +1148,6 @@
           <t>J-2026-2</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr"/>
-      <c r="N9" t="inlineStr"/>
-      <c r="O9" t="inlineStr"/>
       <c r="P9" t="inlineStr">
         <is>
           <t>1</t>
@@ -1167,15 +1158,183 @@
           <t>1</t>
         </is>
       </c>
-      <c r="R9" t="inlineStr"/>
-      <c r="S9" t="inlineStr"/>
-      <c r="T9" t="inlineStr"/>
       <c r="U9" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="V9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>03/05/2026</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>38QRU37D96FM</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Begoña Vázquez Pariente</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>vazquez949@yahoo.es</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>648247065</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Avenida de Castilla, 15</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>4 A</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>19002</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Guadalajara</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Guadalajara</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>2026-05-03 00:00:00</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>JF-2026-1</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr"/>
+      <c r="Q10" t="inlineStr"/>
+      <c r="R10" t="inlineStr"/>
+      <c r="S10" t="inlineStr"/>
+      <c r="T10" t="inlineStr"/>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="V10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>03/05/2026</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>I4QKJ4YFSO8V</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Leticia Vázquez Pariente</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>javier7004@gmail.com</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>692393097</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>París, 208</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>3º 3ª</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>08008</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Barcelona</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Barcelona</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>2026-05-04 00:00:00</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>J-2026-2</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="inlineStr"/>
+      <c r="O11" t="inlineStr"/>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr"/>
+      <c r="S11" t="inlineStr"/>
+      <c r="T11" t="inlineStr"/>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="V11" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update automático: 2026-05-03 20:26
</commit_message>
<xml_diff>
--- a/HISTORICO.xlsx
+++ b/HISTORICO.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V11"/>
+  <dimension ref="A1:V13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1240,17 +1240,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="P10" t="inlineStr"/>
-      <c r="Q10" t="inlineStr"/>
-      <c r="R10" t="inlineStr"/>
-      <c r="S10" t="inlineStr"/>
-      <c r="T10" t="inlineStr"/>
       <c r="U10" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="V10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1313,9 +1307,6 @@
           <t>J-2026-2</t>
         </is>
       </c>
-      <c r="M11" t="inlineStr"/>
-      <c r="N11" t="inlineStr"/>
-      <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr">
         <is>
           <t>1</t>
@@ -1326,15 +1317,183 @@
           <t>1</t>
         </is>
       </c>
-      <c r="R11" t="inlineStr"/>
-      <c r="S11" t="inlineStr"/>
-      <c r="T11" t="inlineStr"/>
       <c r="U11" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="V11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>03/05/2026</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>SPCA4GX5PGQU</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Begoña Vázquez Pariente</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>vazquez949@yahoo.es</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>648247065</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Avenida de Castilla, 15</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>4 A</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>19002</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Guadalajara</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Guadalajara</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>2026-05-03 00:00:00</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>JF-2026-1</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr"/>
+      <c r="Q12" t="inlineStr"/>
+      <c r="R12" t="inlineStr"/>
+      <c r="S12" t="inlineStr"/>
+      <c r="T12" t="inlineStr"/>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="V12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>03/05/2026</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>JNMMS39WA8S3</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Leticia Vázquez Pariente</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>javier7004@gmail.com</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>692393097</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>París, 208</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>3º 3ª</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>08008</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Barcelona</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Barcelona</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>2026-05-04 00:00:00</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>J-2026-2</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="inlineStr"/>
+      <c r="O13" t="inlineStr"/>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr"/>
+      <c r="S13" t="inlineStr"/>
+      <c r="T13" t="inlineStr"/>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="V13" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Actualización automática: 2026-05-04 22:57
</commit_message>
<xml_diff>
--- a/HISTORICO.xlsx
+++ b/HISTORICO.xlsx
@@ -2,15 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -50,7 +49,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -413,8 +412,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V13"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:V22"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
+  <cols>
+    <col width="22.7265625" customWidth="1" min="1" max="1"/>
+    <col width="54.1796875" customWidth="1" min="2" max="2"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -1399,17 +1402,11 @@
           <t>1</t>
         </is>
       </c>
-      <c r="P12" t="inlineStr"/>
-      <c r="Q12" t="inlineStr"/>
-      <c r="R12" t="inlineStr"/>
-      <c r="S12" t="inlineStr"/>
-      <c r="T12" t="inlineStr"/>
       <c r="U12" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="V12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1472,9 +1469,6 @@
           <t>J-2026-2</t>
         </is>
       </c>
-      <c r="M13" t="inlineStr"/>
-      <c r="N13" t="inlineStr"/>
-      <c r="O13" t="inlineStr"/>
       <c r="P13" t="inlineStr">
         <is>
           <t>1</t>
@@ -1485,15 +1479,735 @@
           <t>1</t>
         </is>
       </c>
-      <c r="R13" t="inlineStr"/>
-      <c r="S13" t="inlineStr"/>
-      <c r="T13" t="inlineStr"/>
       <c r="U13" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="V13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Begoña Vázquez Pariente</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>vazquez949@yahoo.es</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>648247065</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Avenida de Castilla, 15</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>4 A</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>19002</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Guadalajara</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Guadalajara</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>2026-05-03 00:00:00</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>JF-2026-1</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>COM407WI5NWV</t>
+        </is>
+      </c>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>03/05/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Leticia Vázquez Pariente</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>javier7004@gmail.com</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>692393097</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>París, 208</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>3º 3ª</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>08008</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Barcelona</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Barcelona</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>2026-05-04 00:00:00</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>J-2026-2</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>SUSKJYH9DVRA</t>
+        </is>
+      </c>
+      <c r="V15" t="inlineStr">
+        <is>
+          <t>03/05/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Begoña Vázquez Pariente</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>vazquez949@yahoo.es</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>648247065</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Avenida de Castilla, 15</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>4 A</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>19002</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Guadalajara</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Guadalajara</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>2026-05-03 00:00:00</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>JF-2026-1</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>COM407WI5NWV</t>
+        </is>
+      </c>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>03/05/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Leticia Vázquez Pariente</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>javier7004@gmail.com</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>692393097</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>París, 208</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>3º 3ª</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>08008</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Barcelona</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Barcelona</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>2026-05-04 00:00:00</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>J-2026-2</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>SUSKJYH9DVRA</t>
+        </is>
+      </c>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t>03/05/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>03/05/2026</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>R64N2AQSDKYX</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Begoña Vázquez Pariente</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>vazquez949@yahoo.es</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>648247065</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Avenida de Castilla, 15</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>4 A</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>19002</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Guadalajara</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>Guadalajara</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>2026-05-03 00:00:00</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>JF-2026-1</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="U18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>03/05/2026</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>4SK5B1UVD903</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Leticia Vázquez Pariente</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>javier7004@gmail.com</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>692393097</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>París, 208</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>3º 3ª</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>08008</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Barcelona</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>Barcelona</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>2026-05-04 00:00:00</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>J-2026-2</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>04/05/2026</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>NPWQUQLA3LDJ</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Begoña Vázquez Pariente</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>vazquez949@yahoo.es</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>648247065</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Avenida de Castilla, 15</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>4 A</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>19002</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Guadalajara</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>Guadalajara</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>2026-05-03 00:00:00</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>JF-2026-1</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="U20" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>04/05/2026</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>7SZH4SM9OB9L</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Leticia Vázquez Pariente</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>javier7004@gmail.com</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>692393097</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>París, 208</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>3º 3ª</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>08008</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Barcelona</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>Barcelona</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>2026-05-04 00:00:00</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>J-2026-2</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="U21" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>04/05/2026</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>WM67HPN0D3HK</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>José María Aznar</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>vazquez949@yahoo.es</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>648247065</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Avenida de Castilla, 15</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>4 A</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>19002</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Guadalajara</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>Guadalajara</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>2026-05-03 00:00:00</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>JF-2026-1</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr"/>
+      <c r="Q22" t="inlineStr"/>
+      <c r="R22" t="inlineStr"/>
+      <c r="S22" t="inlineStr"/>
+      <c r="T22" t="inlineStr"/>
+      <c r="U22" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="V22" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Actualización automática: 2026-05-04 22:59
</commit_message>
<xml_diff>
--- a/HISTORICO.xlsx
+++ b/HISTORICO.xlsx
@@ -412,7 +412,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V22"/>
+  <dimension ref="A1:V23"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <cols>
     <col width="22.7265625" customWidth="1" min="1" max="1"/>
@@ -2197,17 +2197,99 @@
           <t>1</t>
         </is>
       </c>
-      <c r="P22" t="inlineStr"/>
-      <c r="Q22" t="inlineStr"/>
-      <c r="R22" t="inlineStr"/>
-      <c r="S22" t="inlineStr"/>
-      <c r="T22" t="inlineStr"/>
       <c r="U22" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="V22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>04/05/2026</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>QP0404UT25HM</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>José María Aznar</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>vazquez949@yahoo.es</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>648247065</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Avenida de Castilla, 15</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>4 A</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>19002</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Guadalajara</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>Guadalajara</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>2026-05-03 00:00:00</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>JF-2026-1</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr"/>
+      <c r="Q23" t="inlineStr"/>
+      <c r="R23" t="inlineStr"/>
+      <c r="S23" t="inlineStr"/>
+      <c r="T23" t="inlineStr"/>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="V23" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Actualización automática: 2026-05-04 23:12
</commit_message>
<xml_diff>
--- a/HISTORICO.xlsx
+++ b/HISTORICO.xlsx
@@ -412,7 +412,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V23"/>
+  <dimension ref="A1:V24"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <cols>
     <col width="22.7265625" customWidth="1" min="1" max="1"/>
@@ -2279,17 +2279,99 @@
           <t>1</t>
         </is>
       </c>
-      <c r="P23" t="inlineStr"/>
-      <c r="Q23" t="inlineStr"/>
-      <c r="R23" t="inlineStr"/>
-      <c r="S23" t="inlineStr"/>
-      <c r="T23" t="inlineStr"/>
       <c r="U23" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="V23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>04/05/2026</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>EZ8MW7AHNKIG</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>José María Aznar</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>vazquez949@yahoo.es</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>648247065</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Avenida de Castilla, 15</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>4 A</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>19002</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Guadalajara</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>Guadalajara</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>2026-05-03 00:00:00</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>JF-2026-1</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="P24" t="inlineStr"/>
+      <c r="Q24" t="inlineStr"/>
+      <c r="R24" t="inlineStr"/>
+      <c r="S24" t="inlineStr"/>
+      <c r="T24" t="inlineStr"/>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="V24" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Actualización automática: 2026-05-04 23:14
</commit_message>
<xml_diff>
--- a/HISTORICO.xlsx
+++ b/HISTORICO.xlsx
@@ -412,7 +412,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V24"/>
+  <dimension ref="A1:V25"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <cols>
     <col width="22.7265625" customWidth="1" min="1" max="1"/>
@@ -2361,17 +2361,99 @@
           <t>1</t>
         </is>
       </c>
-      <c r="P24" t="inlineStr"/>
-      <c r="Q24" t="inlineStr"/>
-      <c r="R24" t="inlineStr"/>
-      <c r="S24" t="inlineStr"/>
-      <c r="T24" t="inlineStr"/>
       <c r="U24" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="V24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>04/05/2026</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>MEQHKK27MKI2</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>José María Aznar</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>vazquez949@yahoo.es</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>648247065</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Avenida de Castilla, 15</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>4 A</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>19002</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Guadalajara</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>Guadalajara</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>2026-05-03 00:00:00</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>JF-2026-1</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr"/>
+      <c r="Q25" t="inlineStr"/>
+      <c r="R25" t="inlineStr"/>
+      <c r="S25" t="inlineStr"/>
+      <c r="T25" t="inlineStr"/>
+      <c r="U25" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="V25" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>